<commit_message>
checked replies for final outreach reminder
</commit_message>
<xml_diff>
--- a/outputs/200_winners_psid_name_lookup.xlsx
+++ b/outputs/200_winners_psid_name_lookup.xlsx
@@ -648,12 +648,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-06-06T05:48:13+0000</t>
+          <t>2026-06-08T07:19:38+0000</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>87</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -673,21 +673,21 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Tropicana Malaysia</t>
+          <t>Yew Ng</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>594456394024035</t>
+          <t>9706174452773195</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-06-06T05:48:13+0000</t>
+          <t>2026-06-08T07:19:38+0000</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>647</v>
+        <v>16</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -696,13 +696,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Hai Yew Ng,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resit yang...</t>
+          <t>🍊Semak Oren Saya</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
@@ -743,12 +737,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-06-06T05:35:42+0000</t>
+          <t>2026-06-08T08:51:28+0000</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>948</t>
+          <t>955</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -768,21 +762,21 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Tropicana Malaysia</t>
+          <t>Nur Lisya Nadirah</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>594456394024035</t>
+          <t>2412178815500468</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-06-06T05:35:42+0000</t>
+          <t>2026-06-08T08:51:28+0000</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>658</v>
+        <v>34</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -791,13 +785,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Hai Nur Lisya Nadirah,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin...</t>
+          <t>Saya ada 2 resit pembelian produk.</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
@@ -1999,17 +1987,17 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-06-06T09:15:47+0000</t>
+          <t>2026-06-09T13:04:06+0000</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>83</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -2034,11 +2022,11 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-06-06T09:15:47+0000</t>
+          <t>2026-06-09T13:04:06+0000</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2047,7 +2035,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Oraite nnti sy bg details ya</t>
+          <t>Hawatif sent a photo.</t>
         </is>
       </c>
       <c r="S18" t="inlineStr"/>
@@ -2177,12 +2165,12 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-06-06T05:39:12+0000</t>
+          <t>2026-06-08T04:35:12+0000</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>129</t>
+          <t>130</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -2212,11 +2200,11 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-06-06T05:39:12+0000</t>
+          <t>2026-06-08T04:35:12+0000</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>656</v>
+        <v>299</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2226,12 +2214,8 @@
       <c r="R20" t="inlineStr">
         <is>
           <t>Hai Staphyine Cyril,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin r...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak d...</t>
         </is>
       </c>
       <c r="S20" t="inlineStr"/>
@@ -3433,12 +3417,12 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>2026-06-06T05:39:53+0000</t>
+          <t>2026-06-08T04:35:29+0000</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>579</t>
+          <t>580</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -3468,11 +3452,11 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-06-06T05:39:53+0000</t>
+          <t>2026-06-08T04:35:29+0000</t>
         </is>
       </c>
       <c r="P34" t="n">
-        <v>656</v>
+        <v>299</v>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
@@ -3482,12 +3466,8 @@
       <c r="R34" t="inlineStr">
         <is>
           <t>Hai Syaidatul Farah,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin r...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak d...</t>
         </is>
       </c>
       <c r="S34" t="inlineStr"/>
@@ -4426,12 +4406,12 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>2026-06-06T05:27:55+0000</t>
+          <t>2026-06-08T04:27:56+0000</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>179</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4461,11 +4441,11 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-06-06T05:27:55+0000</t>
+          <t>2026-06-08T04:27:56+0000</t>
         </is>
       </c>
       <c r="P45" t="n">
-        <v>651</v>
+        <v>294</v>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
@@ -4475,12 +4455,8 @@
       <c r="R45" t="inlineStr">
         <is>
           <t>Hai Jue Herman,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resit ...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dapat ...</t>
         </is>
       </c>
       <c r="S45" t="inlineStr"/>
@@ -5779,12 +5755,12 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>2026-06-06T05:20:48+0000</t>
+          <t>2026-06-08T04:20:33+0000</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>158</t>
+          <t>159</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -5814,11 +5790,11 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-06-06T05:20:48+0000</t>
+          <t>2026-06-08T04:20:33+0000</t>
         </is>
       </c>
       <c r="P60" t="n">
-        <v>649</v>
+        <v>292</v>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
@@ -5828,12 +5804,8 @@
       <c r="R60" t="inlineStr">
         <is>
           <t>Hai Arni Ani,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resit ya...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dapat di...</t>
         </is>
       </c>
       <c r="S60" t="inlineStr"/>
@@ -6945,12 +6917,12 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>2026-06-06T05:25:07+0000</t>
+          <t>2026-06-08T04:22:41+0000</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>102</t>
+          <t>103</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -6980,11 +6952,11 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-06-06T05:25:07+0000</t>
+          <t>2026-06-08T04:22:41+0000</t>
         </is>
       </c>
       <c r="P73" t="n">
-        <v>653</v>
+        <v>296</v>
       </c>
       <c r="Q73" t="inlineStr">
         <is>
@@ -6994,12 +6966,8 @@
       <c r="R73" t="inlineStr">
         <is>
           <t>Hai Fieyza Peace,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resi...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dapa...</t>
         </is>
       </c>
       <c r="S73" t="inlineStr"/>
@@ -7307,12 +7275,12 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>2026-06-06T05:30:19+0000</t>
+          <t>2026-06-09T06:04:29+0000</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>483</t>
+          <t>488</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -7332,21 +7300,21 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>Tropicana Malaysia</t>
+          <t>Mohamad Azhar Aziz MaxArt</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>594456394024035</t>
+          <t>9536462943096387</t>
         </is>
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-06-06T05:30:19+0000</t>
+          <t>2026-06-09T06:04:29+0000</t>
         </is>
       </c>
       <c r="P77" t="n">
-        <v>666</v>
+        <v>2</v>
       </c>
       <c r="Q77" t="inlineStr">
         <is>
@@ -7355,13 +7323,7 @@
       </c>
       <c r="R77" t="inlineStr">
         <is>
-          <t>Hai Mohamad Azhar Aziz MaxArt,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkap...</t>
+          <t>Tq</t>
         </is>
       </c>
       <c r="S77" t="inlineStr"/>
@@ -7402,12 +7364,12 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>2026-06-06T05:38:49+0000</t>
+          <t>2026-06-08T04:35:02+0000</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>162</t>
+          <t>163</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -7437,11 +7399,11 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-06-06T05:38:49+0000</t>
+          <t>2026-06-08T04:35:02+0000</t>
         </is>
       </c>
       <c r="P78" t="n">
-        <v>667</v>
+        <v>310</v>
       </c>
       <c r="Q78" t="inlineStr">
         <is>
@@ -7451,12 +7413,8 @@
       <c r="R78" t="inlineStr">
         <is>
           <t>Hai Siti Norfqizqh Kqmqruzqmqn,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangka...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah a...</t>
         </is>
       </c>
       <c r="S78" t="inlineStr"/>
@@ -9016,12 +8974,12 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>2026-06-06T05:28:14+0000</t>
+          <t>2026-06-08T04:28:04+0000</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>102</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -9051,11 +9009,11 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>2026-06-06T05:28:14+0000</t>
+          <t>2026-06-08T04:28:04+0000</t>
         </is>
       </c>
       <c r="P96" t="n">
-        <v>653</v>
+        <v>296</v>
       </c>
       <c r="Q96" t="inlineStr">
         <is>
@@ -9065,12 +9023,8 @@
       <c r="R96" t="inlineStr">
         <is>
           <t>Hai Kam Wai Kwan,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resi...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dapa...</t>
         </is>
       </c>
       <c r="S96" t="inlineStr"/>
@@ -9111,12 +9065,12 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>2026-06-06T05:38:17+0000</t>
+          <t>2026-06-08T04:34:43+0000</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>54</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -9146,11 +9100,11 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>2026-06-06T05:38:17+0000</t>
+          <t>2026-06-08T04:34:43+0000</t>
         </is>
       </c>
       <c r="P97" t="n">
-        <v>656</v>
+        <v>299</v>
       </c>
       <c r="Q97" t="inlineStr">
         <is>
@@ -9160,12 +9114,8 @@
       <c r="R97" t="inlineStr">
         <is>
           <t>Hai Shameel Isfahan,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin r...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak d...</t>
         </is>
       </c>
       <c r="S97" t="inlineStr"/>
@@ -9206,12 +9156,12 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>2026-06-06T05:29:06+0000</t>
+          <t>2026-06-08T04:28:37+0000</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>67</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
@@ -9241,11 +9191,11 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>2026-06-06T05:29:06+0000</t>
+          <t>2026-06-08T04:28:37+0000</t>
         </is>
       </c>
       <c r="P98" t="n">
-        <v>653</v>
+        <v>296</v>
       </c>
       <c r="Q98" t="inlineStr">
         <is>
@@ -9255,12 +9205,8 @@
       <c r="R98" t="inlineStr">
         <is>
           <t>Hai Lee Pei Ting,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resi...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dapa...</t>
         </is>
       </c>
       <c r="S98" t="inlineStr"/>
@@ -9390,12 +9336,12 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>2026-06-06T05:38:28+0000</t>
+          <t>2026-06-08T04:34:35+0000</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -9425,11 +9371,11 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>2026-06-06T05:38:28+0000</t>
+          <t>2026-06-08T04:34:35+0000</t>
         </is>
       </c>
       <c r="P100" t="n">
-        <v>656</v>
+        <v>299</v>
       </c>
       <c r="Q100" t="inlineStr">
         <is>
@@ -9439,12 +9385,8 @@
       <c r="R100" t="inlineStr">
         <is>
           <t>Hai Sariffudin Fiza,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin r...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak d...</t>
         </is>
       </c>
       <c r="S100" t="inlineStr"/>
@@ -9666,12 +9608,12 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>2026-06-06T05:41:53+0000</t>
+          <t>2026-06-08T07:08:58+0000</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>74</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -9691,21 +9633,21 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>Tropicana Malaysia</t>
+          <t>JChiang Choon Han</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t>594456394024035</t>
+          <t>25745635091778097</t>
         </is>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>2026-06-06T05:41:53+0000</t>
+          <t>2026-06-08T07:08:58+0000</t>
         </is>
       </c>
       <c r="P103" t="n">
-        <v>658</v>
+        <v>45</v>
       </c>
       <c r="Q103" t="inlineStr">
         <is>
@@ -9714,13 +9656,8 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>Hai JChiang Choon Han,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin...</t>
+          <t>thank you..
+may i know what prize have i won?</t>
         </is>
       </c>
       <c r="S103" t="inlineStr"/>
@@ -9761,12 +9698,12 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>2026-06-06T05:19:57+0000</t>
+          <t>2026-06-08T13:48:03+0000</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>135</t>
+          <t>153</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -9786,21 +9723,21 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>Tropicana Malaysia</t>
+          <t>Alex Chan</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
         <is>
-          <t>594456394024035</t>
+          <t>25787207267568860</t>
         </is>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>2026-06-06T05:19:57+0000</t>
+          <t>2026-06-08T13:48:03+0000</t>
         </is>
       </c>
       <c r="P104" t="n">
-        <v>650</v>
+        <v>4</v>
       </c>
       <c r="Q104" t="inlineStr">
         <is>
@@ -9809,13 +9746,7 @@
       </c>
       <c r="R104" t="inlineStr">
         <is>
-          <t>Hai Alex Chan,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resit y...</t>
+          <t>Ok ?</t>
         </is>
       </c>
       <c r="S104" t="inlineStr"/>
@@ -10034,12 +9965,12 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>2026-06-06T05:25:46+0000</t>
+          <t>2026-06-08T04:58:40+0000</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>53</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
@@ -10069,11 +10000,11 @@
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>2026-06-06T05:25:46+0000</t>
+          <t>2026-06-08T04:58:40+0000</t>
         </is>
       </c>
       <c r="P107" t="n">
-        <v>659</v>
+        <v>43</v>
       </c>
       <c r="Q107" t="inlineStr">
         <is>
@@ -10082,13 +10013,7 @@
       </c>
       <c r="R107" t="inlineStr">
         <is>
-          <t>Hai Himawar Tintin Rie,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skri...</t>
+          <t>Auto-label added: Lead stage set to intake.</t>
         </is>
       </c>
       <c r="S107" t="inlineStr"/>
@@ -10129,12 +10054,12 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>2026-06-06T05:21:22+0000</t>
+          <t>2026-06-08T05:19:44+0000</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
@@ -10154,21 +10079,21 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>Tropicana Malaysia</t>
+          <t>Azi Mah</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
         <is>
-          <t>594456394024035</t>
+          <t>25925220943818297</t>
         </is>
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>2026-06-06T05:21:22+0000</t>
+          <t>2026-06-08T05:19:44+0000</t>
         </is>
       </c>
       <c r="P108" t="n">
-        <v>648</v>
+        <v>11</v>
       </c>
       <c r="Q108" t="inlineStr">
         <is>
@@ -10177,13 +10102,7 @@
       </c>
       <c r="R108" t="inlineStr">
         <is>
-          <t>Hai Azi Mah,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resit yan...</t>
+          <t>Unsubscribe</t>
         </is>
       </c>
       <c r="S108" t="inlineStr"/>
@@ -10313,12 +10232,12 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>2026-06-06T05:42:28+0000</t>
+          <t>2026-06-08T13:18:29+0000</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>52</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
@@ -10338,21 +10257,21 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>Tropicana Malaysia</t>
+          <t>Kavitha Jaganathan</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
         <is>
-          <t>594456394024035</t>
+          <t>25953022347654371</t>
         </is>
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>2026-06-06T05:42:28+0000</t>
+          <t>2026-06-08T13:18:29+0000</t>
         </is>
       </c>
       <c r="P110" t="n">
-        <v>189</v>
+        <v>21</v>
       </c>
       <c r="Q110" t="inlineStr">
         <is>
@@ -10361,9 +10280,7 @@
       </c>
       <c r="R110" t="inlineStr">
         <is>
-          <t>2. Bukti Pembelian
- Gambar atau tangkapan skrin resit yang jelas bersama tarikh dalam Tempoh Promosi.
-sila sertakan resit pembelian Tropicana Twister minimum RM10 untuk melengkapkan syarat</t>
+          <t>Sebab resit dh hilang</t>
         </is>
       </c>
       <c r="S110" t="inlineStr"/>
@@ -10849,12 +10766,12 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>2026-06-06T05:35:54+0000</t>
+          <t>2026-06-08T04:33:15+0000</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
@@ -10884,11 +10801,11 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>2026-06-06T05:35:54+0000</t>
+          <t>2026-06-08T04:33:15+0000</t>
         </is>
       </c>
       <c r="P116" t="n">
-        <v>657</v>
+        <v>300</v>
       </c>
       <c r="Q116" t="inlineStr">
         <is>
@@ -10898,12 +10815,8 @@
       <c r="R116" t="inlineStr">
         <is>
           <t>Hai Nuraina Shahirah,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin ...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak ...</t>
         </is>
       </c>
       <c r="S116" t="inlineStr"/>
@@ -10944,12 +10857,12 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>2026-06-06T05:31:24+0000</t>
+          <t>2026-06-08T04:30:39+0000</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
@@ -10979,11 +10892,11 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>2026-06-06T05:31:24+0000</t>
+          <t>2026-06-08T04:30:39+0000</t>
         </is>
       </c>
       <c r="P117" t="n">
-        <v>652</v>
+        <v>295</v>
       </c>
       <c r="Q117" t="inlineStr">
         <is>
@@ -10993,12 +10906,8 @@
       <c r="R117" t="inlineStr">
         <is>
           <t>Hai Must Leyzha,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resit...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dapat...</t>
         </is>
       </c>
       <c r="S117" t="inlineStr"/>
@@ -11039,12 +10948,12 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>2026-06-06T05:20:08+0000</t>
+          <t>2026-06-08T04:19:57+0000</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
@@ -11074,11 +10983,11 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>2026-06-06T05:20:08+0000</t>
+          <t>2026-06-08T04:19:57+0000</t>
         </is>
       </c>
       <c r="P118" t="n">
-        <v>647</v>
+        <v>290</v>
       </c>
       <c r="Q118" t="inlineStr">
         <is>
@@ -11088,12 +10997,8 @@
       <c r="R118" t="inlineStr">
         <is>
           <t>Hai An Joe,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resit yang...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dapat dipr...</t>
         </is>
       </c>
       <c r="S118" t="inlineStr"/>
@@ -11579,12 +11484,12 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>2026-06-06T05:44:52+0000</t>
+          <t>2026-06-08T14:03:09+0000</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>39</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
@@ -11604,21 +11509,21 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>Tropicana Malaysia</t>
+          <t>Noor Shahirah Othman</t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
         <is>
-          <t>594456394024035</t>
+          <t>26191985463784477</t>
         </is>
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>2026-06-06T05:44:52+0000</t>
+          <t>2026-06-08T14:03:09+0000</t>
         </is>
       </c>
       <c r="P124" t="n">
-        <v>661</v>
+        <v>118</v>
       </c>
       <c r="Q124" t="inlineStr">
         <is>
@@ -11627,13 +11532,9 @@
       </c>
       <c r="R124" t="inlineStr">
         <is>
-          <t>Hai Noor Shahirah Othman,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan sk...</t>
+          <t>Hi Tropicana
+Resit saya dah tak jumpa 
+Dah minta Dekat TF Value Mart, ambil masa , untuk check dengan customer service</t>
         </is>
       </c>
       <c r="S124" t="inlineStr"/>
@@ -11674,12 +11575,12 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>2026-06-06T05:29:30+0000</t>
+          <t>2026-06-08T04:28:46+0000</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
@@ -11709,11 +11610,11 @@
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>2026-06-06T05:29:30+0000</t>
+          <t>2026-06-08T04:28:46+0000</t>
         </is>
       </c>
       <c r="P125" t="n">
-        <v>653</v>
+        <v>296</v>
       </c>
       <c r="Q125" t="inlineStr">
         <is>
@@ -11723,12 +11624,8 @@
       <c r="R125" t="inlineStr">
         <is>
           <t>Hai Lukman Haqem,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resi...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dapa...</t>
         </is>
       </c>
       <c r="S125" t="inlineStr"/>
@@ -11951,12 +11848,12 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>2026-06-06T05:28:44+0000</t>
+          <t>2026-06-08T04:28:26+0000</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
@@ -11986,11 +11883,11 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>2026-06-06T05:28:44+0000</t>
+          <t>2026-06-08T04:28:26+0000</t>
         </is>
       </c>
       <c r="P128" t="n">
-        <v>661</v>
+        <v>304</v>
       </c>
       <c r="Q128" t="inlineStr">
         <is>
@@ -12000,12 +11897,8 @@
       <c r="R128" t="inlineStr">
         <is>
           <t>Hai Kirtanah Ravintharan,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan sk...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda ti...</t>
         </is>
       </c>
       <c r="S128" t="inlineStr"/>
@@ -12672,12 +12565,12 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>2026-06-06T05:21:00+0000</t>
+          <t>2026-06-08T04:20:44+0000</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>94</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -12707,11 +12600,11 @@
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>2026-06-06T05:21:00+0000</t>
+          <t>2026-06-08T04:20:44+0000</t>
         </is>
       </c>
       <c r="P136" t="n">
-        <v>652</v>
+        <v>295</v>
       </c>
       <c r="Q136" t="inlineStr">
         <is>
@@ -12721,12 +12614,8 @@
       <c r="R136" t="inlineStr">
         <is>
           <t>Hai Azfar Azrie,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resit...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dapat...</t>
         </is>
       </c>
       <c r="S136" t="inlineStr"/>
@@ -13039,12 +12928,12 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>2026-06-06T05:37:45+0000</t>
+          <t>2026-06-08T04:34:00+0000</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>411</t>
+          <t>412</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
@@ -13074,11 +12963,11 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>2026-06-06T05:37:45+0000</t>
+          <t>2026-06-08T04:34:00+0000</t>
         </is>
       </c>
       <c r="P140" t="n">
-        <v>653</v>
+        <v>296</v>
       </c>
       <c r="Q140" t="inlineStr">
         <is>
@@ -13088,12 +12977,8 @@
       <c r="R140" t="inlineStr">
         <is>
           <t>Hai Rijah Weiwei,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resi...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dapa...</t>
         </is>
       </c>
       <c r="S140" t="inlineStr"/>
@@ -13134,12 +13019,12 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>2026-06-06T05:39:23+0000</t>
+          <t>2026-06-08T05:34:08+0000</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>89</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
@@ -13159,21 +13044,21 @@
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>Tropicana Malaysia</t>
+          <t>Suhaida M Sobri</t>
         </is>
       </c>
       <c r="N141" t="inlineStr">
         <is>
-          <t>594456394024035</t>
+          <t>26458022533837392</t>
         </is>
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>2026-06-06T05:39:23+0000</t>
+          <t>2026-06-08T05:34:08+0000</t>
         </is>
       </c>
       <c r="P141" t="n">
-        <v>656</v>
+        <v>2</v>
       </c>
       <c r="Q141" t="inlineStr">
         <is>
@@ -13182,13 +13067,7 @@
       </c>
       <c r="R141" t="inlineStr">
         <is>
-          <t>Hai Suhaida M Sobri,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin r...</t>
+          <t>Ok</t>
         </is>
       </c>
       <c r="S141" t="inlineStr"/>
@@ -13318,12 +13197,12 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>2026-06-06T05:30:03+0000</t>
+          <t>2026-06-09T04:22:48+0000</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>89</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
@@ -13353,11 +13232,11 @@
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>2026-06-06T05:30:03+0000</t>
+          <t>2026-06-09T04:22:48+0000</t>
         </is>
       </c>
       <c r="P143" t="n">
-        <v>649</v>
+        <v>43</v>
       </c>
       <c r="Q143" t="inlineStr">
         <is>
@@ -13366,13 +13245,7 @@
       </c>
       <c r="R143" t="inlineStr">
         <is>
-          <t>Hai Miha Mus,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resit ya...</t>
+          <t>Auto-label added: Lead stage set to intake.</t>
         </is>
       </c>
       <c r="S143" t="inlineStr"/>
@@ -13502,12 +13375,12 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>2026-06-06T05:40:39+0000</t>
+          <t>2026-06-08T04:36:05+0000</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
@@ -13537,11 +13410,11 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>2026-06-06T05:40:39+0000</t>
+          <t>2026-06-08T04:36:05+0000</t>
         </is>
       </c>
       <c r="P145" t="n">
-        <v>652</v>
+        <v>295</v>
       </c>
       <c r="Q145" t="inlineStr">
         <is>
@@ -13551,12 +13424,8 @@
       <c r="R145" t="inlineStr">
         <is>
           <t>Hai Ummi Kalsum,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resit...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dapat...</t>
         </is>
       </c>
       <c r="S145" t="inlineStr"/>
@@ -13965,12 +13834,12 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>2026-06-06T05:31:42+0000</t>
+          <t>2026-06-08T04:30:56+0000</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
       <c r="J150" t="inlineStr">
@@ -14000,11 +13869,11 @@
       </c>
       <c r="O150" t="inlineStr">
         <is>
-          <t>2026-06-06T05:31:42+0000</t>
+          <t>2026-06-08T04:30:56+0000</t>
         </is>
       </c>
       <c r="P150" t="n">
-        <v>657</v>
+        <v>300</v>
       </c>
       <c r="Q150" t="inlineStr">
         <is>
@@ -14014,12 +13883,8 @@
       <c r="R150" t="inlineStr">
         <is>
           <t>Hai Nazatul Farhanis,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin ...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak ...</t>
         </is>
       </c>
       <c r="S150" t="inlineStr"/>
@@ -14060,12 +13925,12 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>2026-06-06T05:36:10+0000</t>
+          <t>2026-06-08T04:33:23+0000</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>55</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
@@ -14095,11 +13960,11 @@
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>2026-06-06T05:36:10+0000</t>
+          <t>2026-06-08T04:33:23+0000</t>
         </is>
       </c>
       <c r="P151" t="n">
-        <v>656</v>
+        <v>299</v>
       </c>
       <c r="Q151" t="inlineStr">
         <is>
@@ -14109,12 +13974,8 @@
       <c r="R151" t="inlineStr">
         <is>
           <t>Hai Nurarina Khidir,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin r...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak d...</t>
         </is>
       </c>
       <c r="S151" t="inlineStr"/>
@@ -14155,12 +14016,12 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>2026-06-06T05:29:52+0000</t>
+          <t>2026-06-08T04:29:17+0000</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="J152" t="inlineStr">
@@ -14190,11 +14051,11 @@
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>2026-06-06T05:29:52+0000</t>
+          <t>2026-06-08T04:29:17+0000</t>
         </is>
       </c>
       <c r="P152" t="n">
-        <v>656</v>
+        <v>299</v>
       </c>
       <c r="Q152" t="inlineStr">
         <is>
@@ -14204,12 +14065,8 @@
       <c r="R152" t="inlineStr">
         <is>
           <t>Hai Maria Muhayadin,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin r...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak d...</t>
         </is>
       </c>
       <c r="S152" t="inlineStr"/>
@@ -14339,12 +14196,12 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>2026-06-06T05:21:38+0000</t>
+          <t>2026-06-08T04:21:16+0000</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="J154" t="inlineStr">
@@ -14374,11 +14231,11 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>2026-06-06T05:21:38+0000</t>
+          <t>2026-06-08T04:21:16+0000</t>
         </is>
       </c>
       <c r="P154" t="n">
-        <v>653</v>
+        <v>296</v>
       </c>
       <c r="Q154" t="inlineStr">
         <is>
@@ -14388,12 +14245,8 @@
       <c r="R154" t="inlineStr">
         <is>
           <t>Hai Aziana Nazri,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resi...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dapa...</t>
         </is>
       </c>
       <c r="S154" t="inlineStr"/>
@@ -14434,17 +14287,17 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>2026-06-06T06:23:31+0000</t>
+          <t>2026-06-10T02:13:58+0000</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>72</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
@@ -14469,11 +14322,11 @@
       </c>
       <c r="O155" t="inlineStr">
         <is>
-          <t>2026-06-06T06:23:31+0000</t>
+          <t>2026-06-10T02:13:58+0000</t>
         </is>
       </c>
       <c r="P155" t="n">
-        <v>55</v>
+        <v>187</v>
       </c>
       <c r="Q155" t="inlineStr">
         <is>
@@ -14482,7 +14335,11 @@
       </c>
       <c r="R155" t="inlineStr">
         <is>
-          <t>Jadi boleh buat pembelian baru ya? Ok baik terima kasih</t>
+          <t>Maklumat Peribadi
+ Nama penuh (seperti dalam IC): AIDA NATASHA 
+ No. IC: 000628-10-1318
+ No. Telefon: 0173501169
+ Alamat Penghantaran: NO 67 JALAN ENGGANG TAMAN KERAMAT 54200 Kuala LUMPUR</t>
         </is>
       </c>
       <c r="S155" t="inlineStr"/>
@@ -14523,12 +14380,12 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>2026-06-06T05:35:28+0000</t>
+          <t>2026-06-08T04:32:54+0000</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
@@ -14558,11 +14415,11 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>2026-06-06T05:35:28+0000</t>
+          <t>2026-06-08T04:32:54+0000</t>
         </is>
       </c>
       <c r="P156" t="n">
-        <v>658</v>
+        <v>301</v>
       </c>
       <c r="Q156" t="inlineStr">
         <is>
@@ -14572,12 +14429,8 @@
       <c r="R156" t="inlineStr">
         <is>
           <t>Hai Nur Kiawati Wahib,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak...</t>
         </is>
       </c>
       <c r="S156" t="inlineStr"/>
@@ -14618,12 +14471,12 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>2026-06-06T05:40:04+0000</t>
+          <t>2026-06-08T04:35:38+0000</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>36</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
@@ -14653,11 +14506,11 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>2026-06-06T05:40:04+0000</t>
+          <t>2026-06-08T04:35:38+0000</t>
         </is>
       </c>
       <c r="P157" t="n">
-        <v>654</v>
+        <v>297</v>
       </c>
       <c r="Q157" t="inlineStr">
         <is>
@@ -14667,12 +14520,8 @@
       <c r="R157" t="inlineStr">
         <is>
           <t>Hai Syikin Supian,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin res...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dap...</t>
         </is>
       </c>
       <c r="S157" t="inlineStr"/>
@@ -14802,12 +14651,12 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>2026-06-06T05:30:37+0000</t>
+          <t>2026-06-09T09:53:10+0000</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>35</t>
         </is>
       </c>
       <c r="J159" t="inlineStr">
@@ -14827,21 +14676,21 @@
       </c>
       <c r="M159" t="inlineStr">
         <is>
-          <t>Tropicana Malaysia</t>
+          <t>Mohd Khairul Hafiz</t>
         </is>
       </c>
       <c r="N159" t="inlineStr">
         <is>
-          <t>594456394024035</t>
+          <t>26655419207422712</t>
         </is>
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>2026-06-06T05:30:37+0000</t>
+          <t>2026-06-09T09:53:10+0000</t>
         </is>
       </c>
       <c r="P159" t="n">
-        <v>659</v>
+        <v>11</v>
       </c>
       <c r="Q159" t="inlineStr">
         <is>
@@ -14850,13 +14699,7 @@
       </c>
       <c r="R159" t="inlineStr">
         <is>
-          <t>Hai Mohd Khairul Hafiz,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skri...</t>
+          <t>Done hantar</t>
         </is>
       </c>
       <c r="S159" t="inlineStr"/>
@@ -14986,12 +14829,12 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>2026-06-06T05:25:17+0000</t>
+          <t>2026-06-08T04:22:51+0000</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
@@ -15021,11 +14864,11 @@
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>2026-06-06T05:25:17+0000</t>
+          <t>2026-06-08T04:22:51+0000</t>
         </is>
       </c>
       <c r="P161" t="n">
-        <v>655</v>
+        <v>298</v>
       </c>
       <c r="Q161" t="inlineStr">
         <is>
@@ -15035,12 +14878,8 @@
       <c r="R161" t="inlineStr">
         <is>
           <t>Hai Firdaus Hakimi,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin re...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak da...</t>
         </is>
       </c>
       <c r="S161" t="inlineStr"/>
@@ -15081,12 +14920,12 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>2026-06-06T05:26:49+0000</t>
+          <t>2026-06-08T04:27:25+0000</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>284</t>
+          <t>285</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
@@ -15116,11 +14955,11 @@
       </c>
       <c r="O162" t="inlineStr">
         <is>
-          <t>2026-06-06T05:26:49+0000</t>
+          <t>2026-06-08T04:27:25+0000</t>
         </is>
       </c>
       <c r="P162" t="n">
-        <v>654</v>
+        <v>297</v>
       </c>
       <c r="Q162" t="inlineStr">
         <is>
@@ -15130,12 +14969,8 @@
       <c r="R162" t="inlineStr">
         <is>
           <t>Hai Ikhwan Shafiq,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin res...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dap...</t>
         </is>
       </c>
       <c r="S162" t="inlineStr"/>
@@ -15176,12 +15011,12 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>2026-06-06T05:36:27+0000</t>
+          <t>2026-06-08T04:33:32+0000</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>55</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
@@ -15211,11 +15046,11 @@
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>2026-06-06T05:36:27+0000</t>
+          <t>2026-06-08T04:33:32+0000</t>
         </is>
       </c>
       <c r="P163" t="n">
-        <v>662</v>
+        <v>305</v>
       </c>
       <c r="Q163" t="inlineStr">
         <is>
@@ -15225,12 +15060,8 @@
       <c r="R163" t="inlineStr">
         <is>
           <t>Hai Nurnadia Kamaruzzaman,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan s...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda t...</t>
         </is>
       </c>
       <c r="S163" t="inlineStr"/>
@@ -15271,12 +15102,12 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>2026-06-06T05:34:24+0000</t>
+          <t>2026-06-08T05:31:16+0000</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>63</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
@@ -15306,11 +15137,11 @@
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>2026-06-06T05:34:24+0000</t>
+          <t>2026-06-08T05:31:16+0000</t>
         </is>
       </c>
       <c r="P164" t="n">
-        <v>660</v>
+        <v>52</v>
       </c>
       <c r="Q164" t="inlineStr">
         <is>
@@ -15319,13 +15150,7 @@
       </c>
       <c r="R164" t="inlineStr">
         <is>
-          <t>Hai Nor Azlina Abdullah,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skr...</t>
+          <t>boleh beli baru dan share resit di sini minimum RM10</t>
         </is>
       </c>
       <c r="S164" t="inlineStr"/>
@@ -15366,12 +15191,12 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>2026-06-06T05:24:46+0000</t>
+          <t>2026-06-08T04:22:20+0000</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
@@ -15401,11 +15226,11 @@
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>2026-06-06T05:24:46+0000</t>
+          <t>2026-06-08T04:22:20+0000</t>
         </is>
       </c>
       <c r="P165" t="n">
-        <v>656</v>
+        <v>299</v>
       </c>
       <c r="Q165" t="inlineStr">
         <is>
@@ -15415,12 +15240,8 @@
       <c r="R165" t="inlineStr">
         <is>
           <t>Hai Fendi Zainuddin,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin r...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak d...</t>
         </is>
       </c>
       <c r="S165" t="inlineStr"/>
@@ -15554,12 +15375,12 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>2026-06-06T05:38:00+0000</t>
+          <t>2026-06-08T04:34:12+0000</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
@@ -15589,11 +15410,11 @@
       </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t>2026-06-06T05:38:00+0000</t>
+          <t>2026-06-08T04:34:12+0000</t>
         </is>
       </c>
       <c r="P167" t="n">
-        <v>654</v>
+        <v>297</v>
       </c>
       <c r="Q167" t="inlineStr">
         <is>
@@ -15603,12 +15424,8 @@
       <c r="R167" t="inlineStr">
         <is>
           <t>Hai Salmah Jaafar,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin res...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dap...</t>
         </is>
       </c>
       <c r="S167" t="inlineStr"/>
@@ -15649,12 +15466,12 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>2026-06-06T05:34:12+0000</t>
+          <t>2026-06-08T04:31:37+0000</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>64</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
@@ -15684,11 +15501,11 @@
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>2026-06-06T05:34:12+0000</t>
+          <t>2026-06-08T04:31:37+0000</t>
         </is>
       </c>
       <c r="P168" t="n">
-        <v>654</v>
+        <v>297</v>
       </c>
       <c r="Q168" t="inlineStr">
         <is>
@@ -15698,12 +15515,8 @@
       <c r="R168" t="inlineStr">
         <is>
           <t>Hai Noor Akmawati,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin res...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dap...</t>
         </is>
       </c>
       <c r="S168" t="inlineStr"/>
@@ -15744,12 +15557,12 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>2026-06-06T05:31:10+0000</t>
+          <t>2026-06-08T04:30:15+0000</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>45</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
@@ -15779,11 +15592,11 @@
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>2026-06-06T05:31:10+0000</t>
+          <t>2026-06-08T04:30:15+0000</t>
         </is>
       </c>
       <c r="P169" t="n">
-        <v>669</v>
+        <v>312</v>
       </c>
       <c r="Q169" t="inlineStr">
         <is>
@@ -15793,12 +15606,8 @@
       <c r="R169" t="inlineStr">
         <is>
           <t>Hai Muhammad Zazmie Bin Amirudin,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tang...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah...</t>
         </is>
       </c>
       <c r="S169" t="inlineStr"/>
@@ -15930,12 +15739,12 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>2026-06-06T05:38:39+0000</t>
+          <t>2026-06-08T04:34:52+0000</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>37</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
@@ -15965,11 +15774,11 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>2026-06-06T05:38:39+0000</t>
+          <t>2026-06-08T04:34:52+0000</t>
         </is>
       </c>
       <c r="P171" t="n">
-        <v>654</v>
+        <v>297</v>
       </c>
       <c r="Q171" t="inlineStr">
         <is>
@@ -15979,12 +15788,8 @@
       <c r="R171" t="inlineStr">
         <is>
           <t>Hai Shazlin Rosly,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin res...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dap...</t>
         </is>
       </c>
       <c r="S171" t="inlineStr"/>
@@ -16025,12 +15830,12 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>2026-06-06T05:26:28+0000</t>
+          <t>2026-06-08T04:27:11+0000</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
@@ -16060,11 +15865,11 @@
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>2026-06-06T05:26:28+0000</t>
+          <t>2026-06-08T04:27:11+0000</t>
         </is>
       </c>
       <c r="P172" t="n">
-        <v>651</v>
+        <v>294</v>
       </c>
       <c r="Q172" t="inlineStr">
         <is>
@@ -16074,12 +15879,8 @@
       <c r="R172" t="inlineStr">
         <is>
           <t>Hai Idha Idris,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resit ...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dapat ...</t>
         </is>
       </c>
       <c r="S172" t="inlineStr"/>
@@ -16120,12 +15921,12 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>2026-06-06T05:24:29+0000</t>
+          <t>2026-06-08T04:22:10+0000</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>46</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
@@ -16155,11 +15956,11 @@
       </c>
       <c r="O173" t="inlineStr">
         <is>
-          <t>2026-06-06T05:24:29+0000</t>
+          <t>2026-06-08T04:22:10+0000</t>
         </is>
       </c>
       <c r="P173" t="n">
-        <v>651</v>
+        <v>294</v>
       </c>
       <c r="Q173" t="inlineStr">
         <is>
@@ -16169,12 +15970,8 @@
       <c r="R173" t="inlineStr">
         <is>
           <t>Hai Fairous BI,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resit ...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dapat ...</t>
         </is>
       </c>
       <c r="S173" t="inlineStr"/>
@@ -16215,12 +16012,12 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>2026-06-06T05:28:34+0000</t>
+          <t>2026-06-08T04:28:16+0000</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>92</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
@@ -16250,11 +16047,11 @@
       </c>
       <c r="O174" t="inlineStr">
         <is>
-          <t>2026-06-06T05:28:34+0000</t>
+          <t>2026-06-08T04:28:16+0000</t>
         </is>
       </c>
       <c r="P174" t="n">
-        <v>657</v>
+        <v>300</v>
       </c>
       <c r="Q174" t="inlineStr">
         <is>
@@ -16264,12 +16061,8 @@
       <c r="R174" t="inlineStr">
         <is>
           <t>Hai Khawlah Al Azwar,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin ...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak ...</t>
         </is>
       </c>
       <c r="S174" t="inlineStr"/>
@@ -16399,12 +16192,12 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>2026-06-06T05:22:03+0000</t>
+          <t>2026-06-08T04:21:45+0000</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
@@ -16434,11 +16227,11 @@
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t>2026-06-06T05:22:03+0000</t>
+          <t>2026-06-08T04:21:45+0000</t>
         </is>
       </c>
       <c r="P176" t="n">
-        <v>647</v>
+        <v>290</v>
       </c>
       <c r="Q176" t="inlineStr">
         <is>
@@ -16448,12 +16241,8 @@
       <c r="R176" t="inlineStr">
         <is>
           <t>Hai Ct Ayu,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resit yang...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dapat dipr...</t>
         </is>
       </c>
       <c r="S176" t="inlineStr"/>
@@ -16494,12 +16283,12 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>2026-06-06T05:34:35+0000</t>
+          <t>2026-06-08T04:32:21+0000</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>62</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
@@ -16529,11 +16318,11 @@
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t>2026-06-06T05:34:35+0000</t>
+          <t>2026-06-08T04:32:21+0000</t>
         </is>
       </c>
       <c r="P177" t="n">
-        <v>664</v>
+        <v>307</v>
       </c>
       <c r="Q177" t="inlineStr">
         <is>
@@ -16543,12 +16332,8 @@
       <c r="R177" t="inlineStr">
         <is>
           <t>Hai Normah Hussin Snowwhite,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda...</t>
         </is>
       </c>
       <c r="S177" t="inlineStr"/>
@@ -16678,12 +16463,12 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>2026-06-06T05:19:47+0000</t>
+          <t>2026-06-08T04:19:35+0000</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>39</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
@@ -16713,11 +16498,11 @@
       </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>2026-06-06T05:19:47+0000</t>
+          <t>2026-06-08T04:19:35+0000</t>
         </is>
       </c>
       <c r="P179" t="n">
-        <v>654</v>
+        <v>297</v>
       </c>
       <c r="Q179" t="inlineStr">
         <is>
@@ -16727,12 +16512,8 @@
       <c r="R179" t="inlineStr">
         <is>
           <t>Hai Aizat Kun Kap,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin res...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dap...</t>
         </is>
       </c>
       <c r="S179" t="inlineStr"/>
@@ -16773,12 +16554,12 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>2026-06-06T05:25:33+0000</t>
+          <t>2026-06-08T04:23:01+0000</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>67</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
@@ -16808,11 +16589,11 @@
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>2026-06-06T05:25:33+0000</t>
+          <t>2026-06-08T04:23:01+0000</t>
         </is>
       </c>
       <c r="P180" t="n">
-        <v>667</v>
+        <v>310</v>
       </c>
       <c r="Q180" t="inlineStr">
         <is>
@@ -16822,12 +16603,8 @@
       <c r="R180" t="inlineStr">
         <is>
           <t>Hai Hazirah Manies Haji Johari,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangka...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah a...</t>
         </is>
       </c>
       <c r="S180" t="inlineStr"/>
@@ -16868,12 +16645,12 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>2026-06-06T05:32:31+0000</t>
+          <t>2026-06-08T04:31:22+0000</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>48</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
@@ -16903,11 +16680,11 @@
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>2026-06-06T05:32:31+0000</t>
+          <t>2026-06-08T04:31:22+0000</t>
         </is>
       </c>
       <c r="P181" t="n">
-        <v>649</v>
+        <v>292</v>
       </c>
       <c r="Q181" t="inlineStr">
         <is>
@@ -16917,12 +16694,8 @@
       <c r="R181" t="inlineStr">
         <is>
           <t>Hai Nisya MK,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resit ya...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dapat di...</t>
         </is>
       </c>
       <c r="S181" t="inlineStr"/>
@@ -16963,12 +16736,12 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>2026-06-06T05:24:55+0000</t>
+          <t>2026-06-08T04:23:35+0000</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>53</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
@@ -16988,21 +16761,21 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>Tropicana Malaysia</t>
+          <t>Fezy Lah Deen</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
         <is>
-          <t>594456394024035</t>
+          <t>27642021585386706</t>
         </is>
       </c>
       <c r="O182" t="inlineStr">
         <is>
-          <t>2026-06-06T05:24:55+0000</t>
+          <t>2026-06-08T04:23:35+0000</t>
         </is>
       </c>
       <c r="P182" t="n">
-        <v>654</v>
+        <v>8</v>
       </c>
       <c r="Q182" t="inlineStr">
         <is>
@@ -17011,13 +16784,7 @@
       </c>
       <c r="R182" t="inlineStr">
         <is>
-          <t>Hai Fezy Lah Deen,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin res...</t>
+          <t>Ok noted</t>
         </is>
       </c>
       <c r="S182" t="inlineStr"/>
@@ -17414,12 +17181,12 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>2026-06-06T05:41:02+0000</t>
+          <t>2026-06-08T04:36:14+0000</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
@@ -17449,11 +17216,11 @@
       </c>
       <c r="O187" t="inlineStr">
         <is>
-          <t>2026-06-06T05:41:02+0000</t>
+          <t>2026-06-08T04:36:14+0000</t>
         </is>
       </c>
       <c r="P187" t="n">
-        <v>651</v>
+        <v>294</v>
       </c>
       <c r="Q187" t="inlineStr">
         <is>
@@ -17463,12 +17230,8 @@
       <c r="R187" t="inlineStr">
         <is>
           <t>Hai Wan Aisyah,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resit ...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dapat ...</t>
         </is>
       </c>
       <c r="S187" t="inlineStr"/>
@@ -17687,12 +17450,12 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>2026-06-06T05:35:09+0000</t>
+          <t>2026-06-08T04:32:47+0000</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>56</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
@@ -17722,11 +17485,11 @@
       </c>
       <c r="O190" t="inlineStr">
         <is>
-          <t>2026-06-06T05:35:09+0000</t>
+          <t>2026-06-08T04:32:47+0000</t>
         </is>
       </c>
       <c r="P190" t="n">
-        <v>652</v>
+        <v>295</v>
       </c>
       <c r="Q190" t="inlineStr">
         <is>
@@ -17736,12 +17499,8 @@
       <c r="R190" t="inlineStr">
         <is>
           <t>Hai Nur Hidayah,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resit...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dapat...</t>
         </is>
       </c>
       <c r="S190" t="inlineStr"/>
@@ -17782,12 +17541,12 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>2026-06-06T05:23:51+0000</t>
+          <t>2026-06-09T08:16:44+0000</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>371</t>
+          <t>377</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
@@ -17807,21 +17566,21 @@
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>Tropicana Malaysia</t>
+          <t>Eizec Harith</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">
         <is>
-          <t>594456394024035</t>
+          <t>34683450771303418</t>
         </is>
       </c>
       <c r="O191" t="inlineStr">
         <is>
-          <t>2026-06-06T05:23:51+0000</t>
+          <t>2026-06-09T08:16:44+0000</t>
         </is>
       </c>
       <c r="P191" t="n">
-        <v>653</v>
+        <v>83</v>
       </c>
       <c r="Q191" t="inlineStr">
         <is>
@@ -17830,13 +17589,8 @@
       </c>
       <c r="R191" t="inlineStr">
         <is>
-          <t>Hai Eizec Harith,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resi...</t>
+          <t>Hi ive provided the details before the dateline
+I will still get the reward right?</t>
         </is>
       </c>
       <c r="S191" t="inlineStr"/>
@@ -17877,12 +17631,12 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>2026-06-06T05:20:23+0000</t>
+          <t>2026-06-08T04:20:10+0000</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>59</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
@@ -17912,11 +17666,11 @@
       </c>
       <c r="O192" t="inlineStr">
         <is>
-          <t>2026-06-06T05:20:23+0000</t>
+          <t>2026-06-08T04:20:10+0000</t>
         </is>
       </c>
       <c r="P192" t="n">
-        <v>652</v>
+        <v>295</v>
       </c>
       <c r="Q192" t="inlineStr">
         <is>
@@ -17926,12 +17680,8 @@
       <c r="R192" t="inlineStr">
         <is>
           <t>Hai Angah Angah,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resit...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dapat...</t>
         </is>
       </c>
       <c r="S192" t="inlineStr"/>
@@ -17972,12 +17722,12 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>2026-06-06T05:21:49+0000</t>
+          <t>2026-06-08T04:21:35+0000</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
@@ -18007,11 +17757,11 @@
       </c>
       <c r="O193" t="inlineStr">
         <is>
-          <t>2026-06-06T05:21:49+0000</t>
+          <t>2026-06-08T04:21:35+0000</t>
         </is>
       </c>
       <c r="P193" t="n">
-        <v>655</v>
+        <v>298</v>
       </c>
       <c r="Q193" t="inlineStr">
         <is>
@@ -18021,12 +17771,8 @@
       <c r="R193" t="inlineStr">
         <is>
           <t>Hai Azli Abd Rahim,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin re...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak da...</t>
         </is>
       </c>
       <c r="S193" t="inlineStr"/>
@@ -18067,12 +17813,12 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>2026-06-06T05:15:32+0000</t>
+          <t>2026-06-09T10:06:33+0000</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>356</t>
+          <t>361</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
@@ -18092,21 +17838,21 @@
       </c>
       <c r="M194" t="inlineStr">
         <is>
-          <t>Tropicana Malaysia</t>
+          <t>Afiq Fariz</t>
         </is>
       </c>
       <c r="N194" t="inlineStr">
         <is>
-          <t>594456394024035</t>
+          <t>34935708949349416</t>
         </is>
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>2026-06-06T05:15:32+0000</t>
+          <t>2026-06-09T10:06:33+0000</t>
         </is>
       </c>
       <c r="P194" t="n">
-        <v>651</v>
+        <v>0</v>
       </c>
       <c r="Q194" t="inlineStr">
         <is>
@@ -18115,13 +17861,7 @@
       </c>
       <c r="R194" t="inlineStr">
         <is>
-          <t>Hai Afiq Fariz,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resit ...</t>
+          <t>Afiq sent a photo.</t>
         </is>
       </c>
       <c r="S194" t="inlineStr"/>
@@ -18162,12 +17902,12 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>2026-06-06T05:20:37+0000</t>
+          <t>2026-06-08T04:20:22+0000</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
@@ -18197,11 +17937,11 @@
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t>2026-06-06T05:20:37+0000</t>
+          <t>2026-06-08T04:20:22+0000</t>
         </is>
       </c>
       <c r="P195" t="n">
-        <v>648</v>
+        <v>291</v>
       </c>
       <c r="Q195" t="inlineStr">
         <is>
@@ -18211,12 +17951,8 @@
       <c r="R195" t="inlineStr">
         <is>
           <t>Hai ARe Jim,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resit yan...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dapat dip...</t>
         </is>
       </c>
       <c r="S195" t="inlineStr"/>
@@ -18257,12 +17993,12 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>2026-06-06T05:34:48+0000</t>
+          <t>2026-06-10T02:32:04+0000</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>193</t>
         </is>
       </c>
       <c r="J196" t="inlineStr">
@@ -18282,21 +18018,21 @@
       </c>
       <c r="M196" t="inlineStr">
         <is>
-          <t>Tropicana Malaysia</t>
+          <t>Nur Abas</t>
         </is>
       </c>
       <c r="N196" t="inlineStr">
         <is>
-          <t>594456394024035</t>
+          <t>34997155886550414</t>
         </is>
       </c>
       <c r="O196" t="inlineStr">
         <is>
-          <t>2026-06-06T05:34:48+0000</t>
+          <t>2026-06-10T02:32:04+0000</t>
         </is>
       </c>
       <c r="P196" t="n">
-        <v>649</v>
+        <v>36</v>
       </c>
       <c r="Q196" t="inlineStr">
         <is>
@@ -18305,13 +18041,7 @@
       </c>
       <c r="R196" t="inlineStr">
         <is>
-          <t>Hai Nur Abas,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin resit ya...</t>
+          <t>bole hantar lagi ke dan resit hilang</t>
         </is>
       </c>
       <c r="S196" t="inlineStr"/>
@@ -18352,12 +18082,12 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>2026-06-06T05:37:29+0000</t>
+          <t>2026-06-08T04:33:53+0000</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>48</t>
         </is>
       </c>
       <c r="J197" t="inlineStr">
@@ -18387,11 +18117,11 @@
       </c>
       <c r="O197" t="inlineStr">
         <is>
-          <t>2026-06-06T05:37:29+0000</t>
+          <t>2026-06-08T04:33:53+0000</t>
         </is>
       </c>
       <c r="P197" t="n">
-        <v>657</v>
+        <v>300</v>
       </c>
       <c r="Q197" t="inlineStr">
         <is>
@@ -18401,12 +18131,8 @@
       <c r="R197" t="inlineStr">
         <is>
           <t>Hai Rasidah Rosmanan,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin ...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak ...</t>
         </is>
       </c>
       <c r="S197" t="inlineStr"/>
@@ -18536,12 +18262,12 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>2026-06-06T05:37:01+0000</t>
+          <t>2026-06-08T04:33:40+0000</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>39</t>
         </is>
       </c>
       <c r="J199" t="inlineStr">
@@ -18571,11 +18297,11 @@
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>2026-06-06T05:37:01+0000</t>
+          <t>2026-06-08T04:33:40+0000</t>
         </is>
       </c>
       <c r="P199" t="n">
-        <v>654</v>
+        <v>297</v>
       </c>
       <c r="Q199" t="inlineStr">
         <is>
@@ -18585,12 +18311,8 @@
       <c r="R199" t="inlineStr">
         <is>
           <t>Hai Nurul Knewrul,
-Peringatan untuk hantar maklumat anda sebelum 10 Jun 2026, 8pm bagi meneruskan proses penebusan hadiah.
-Nama Penuh (seperti dalam IC):
-No. IC:
-No. Telefon:
-Alamat Penghantaran:
-2. Bukti Pembelian* Gambar atau tangkapan skrin res...</t>
+Ini adalah peringatan terakhir untuk menghantar maklumat yang diperlukan sebelum 9 Jun 2026, jam 8 malam bagi tujuan penebusan hadiah anda.
+Sekiranya maklumat tidak diterima sebelum tarikh dan masa tersebut, hadiah anda tidak dap...</t>
         </is>
       </c>
       <c r="S199" t="inlineStr"/>

</xml_diff>